<commit_message>
Updated Manual, NW_design, and configmap
</commit_message>
<xml_diff>
--- a/docs/Design/NW/NW_design_tf.xlsx
+++ b/docs/Design/NW/NW_design_tf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ryota/Documents/研鑽/技術/Projects/20250110_KubernetesAPI/graphapp/docs/Design/NW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49496245-6004-9F41-A00C-EA4DE97B7A06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF1CB764-DDA4-664F-BD1E-1AE41CE2F5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1400" yWindow="540" windowWidth="29320" windowHeight="19660" xr2:uid="{A262E15D-8A74-E342-96E0-9E111D7ACA0C}"/>
+    <workbookView xWindow="16360" yWindow="660" windowWidth="16040" windowHeight="20180" activeTab="2" xr2:uid="{A262E15D-8A74-E342-96E0-9E111D7ACA0C}"/>
   </bookViews>
   <sheets>
     <sheet name="System Architecture" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="36">
   <si>
     <t>System Architecture</t>
   </si>
@@ -148,6 +147,11 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>80
+3000
+8080</t>
   </si>
 </sst>
 </file>
@@ -4895,8 +4899,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="3637659" y="3708871"/>
-          <a:ext cx="1198227" cy="2916983"/>
+          <a:off x="3618417" y="3612038"/>
+          <a:ext cx="1190158" cy="2821392"/>
           <a:chOff x="1019709" y="3680217"/>
           <a:chExt cx="1195839" cy="2808833"/>
         </a:xfrm>
@@ -5254,8 +5258,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="6073581" y="3699601"/>
-          <a:ext cx="1198226" cy="2916983"/>
+          <a:off x="6030130" y="3602768"/>
+          <a:ext cx="1190157" cy="2821392"/>
           <a:chOff x="1019709" y="3680216"/>
           <a:chExt cx="1195840" cy="2808832"/>
         </a:xfrm>
@@ -6925,8 +6929,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="2376518" y="6007874"/>
-          <a:ext cx="1043245" cy="821268"/>
+          <a:off x="2373414" y="5835934"/>
+          <a:ext cx="1027107" cy="793956"/>
           <a:chOff x="2356588" y="5815450"/>
           <a:chExt cx="1036373" cy="791030"/>
         </a:xfrm>
@@ -7235,8 +7239,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7584287" y="5983629"/>
-          <a:ext cx="1047095" cy="821268"/>
+          <a:off x="7524698" y="5811689"/>
+          <a:ext cx="1039025" cy="793956"/>
           <a:chOff x="7540305" y="5791205"/>
           <a:chExt cx="1043658" cy="791030"/>
         </a:xfrm>
@@ -10152,7 +10156,7 @@
         <v>8</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="L3" s="7" t="s">
         <v>29</v>

</xml_diff>